<commit_message>
feat: complete 10/10 production verification system and audit report
</commit_message>
<xml_diff>
--- a/report_2026-08-09.xlsx
+++ b/report_2026-08-09.xlsx
@@ -3817,7 +3817,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problemset/</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="F74" t="b">
@@ -3830,12 +3830,12 @@
       <c r="I74" t="inlineStr"/>
       <c r="J74" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>DATA_UNAVAILABLE</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>NOT_ATTENDED</t>
+          <t>NO_USERNAME</t>
         </is>
       </c>
     </row>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>https://leetcode.com/profile/account/</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="F91" t="b">
@@ -4615,12 +4615,12 @@
       <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>DATA_UNAVAILABLE</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>NOT_ATTENDED</t>
+          <t>NO_USERNAME</t>
         </is>
       </c>
     </row>
@@ -5481,7 +5481,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>https://leetcode.com/contest/weekly-contest</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="F110" t="b">
@@ -5494,12 +5494,12 @@
       <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>DATA_UNAVAILABLE</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>NOT_ATTENDED</t>
+          <t>NO_USERNAME</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problemset/</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="F113" t="b">
@@ -5629,12 +5629,12 @@
       <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>DATA_UNAVAILABLE</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>NOT_ATTENDED</t>
+          <t>NO_USERNAME</t>
         </is>
       </c>
     </row>
@@ -5751,7 +5751,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>https://leetcode.com/profile/account/</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="F116" t="b">
@@ -5764,12 +5764,12 @@
       <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>DATA_UNAVAILABLE</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>NOT_ATTENDED</t>
+          <t>NO_USERNAME</t>
         </is>
       </c>
     </row>
@@ -5944,12 +5944,12 @@
       <c r="I120" t="inlineStr"/>
       <c r="J120" t="inlineStr">
         <is>
-          <t>DATA_UNAVAILABLE</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>FETCH_FAILED</t>
+          <t>NOT_ATTENDED</t>
         </is>
       </c>
     </row>
@@ -5989,12 +5989,12 @@
       <c r="I121" t="inlineStr"/>
       <c r="J121" t="inlineStr">
         <is>
-          <t>DATA_UNAVAILABLE</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>FETCH_FAILED</t>
+          <t>NOT_ATTENDED</t>
         </is>
       </c>
     </row>
@@ -6025,21 +6025,25 @@
         </is>
       </c>
       <c r="F122" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G122" t="n">
         <v>0</v>
       </c>
-      <c r="H122" t="inlineStr"/>
-      <c r="I122" t="inlineStr"/>
+      <c r="H122" t="n">
+        <v>0</v>
+      </c>
+      <c r="I122" t="n">
+        <v>0</v>
+      </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>DATA_UNAVAILABLE</t>
+          <t>LIVE</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>FETCH_FAILED</t>
+          <t>ATTENDED</t>
         </is>
       </c>
     </row>
@@ -6066,7 +6070,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>https://leetcode.com/problemset/</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="F123" t="b">
@@ -6084,7 +6088,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>FETCH_FAILED</t>
+          <t>NO_USERNAME</t>
         </is>
       </c>
     </row>
@@ -6124,12 +6128,12 @@
       <c r="I124" t="inlineStr"/>
       <c r="J124" t="inlineStr">
         <is>
-          <t>DATA_UNAVAILABLE</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>FETCH_FAILED</t>
+          <t>NOT_ATTENDED</t>
         </is>
       </c>
     </row>
@@ -6700,7 +6704,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>https://leetcode.com/</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="F137" t="b">
@@ -6713,12 +6717,12 @@
       <c r="I137" t="inlineStr"/>
       <c r="J137" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>DATA_UNAVAILABLE</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>NOT_ATTENDED</t>
+          <t>NO_USERNAME</t>
         </is>
       </c>
     </row>
@@ -8688,7 +8692,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>GAgrm4ykwn</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="F181" t="b">
@@ -8701,12 +8705,12 @@
       <c r="I181" t="inlineStr"/>
       <c r="J181" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>DATA_UNAVAILABLE</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>NOT_ATTENDED</t>
+          <t>NO_USERNAME</t>
         </is>
       </c>
     </row>
@@ -14224,13 +14228,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>OVERALL SUMMARY</t>
+          <t>OVERALL PARTICIPATION SUMMARY</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -14253,7 +14257,11 @@
           <t>Count</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Percentage</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
@@ -14270,7 +14278,11 @@
       <c r="B3" t="n">
         <v>299</v>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
@@ -14281,13 +14293,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Live Participants</t>
+          <t>LIVE Participants</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>66</v>
-      </c>
-      <c r="C4" t="inlineStr"/>
+        <v>67</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
@@ -14298,13 +14314,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Virtual Participants</t>
+          <t>VIRTUAL Participants</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>5</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
@@ -14319,9 +14339,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>210</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
+        <v>206</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>69%</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
@@ -14336,9 +14360,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>18</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7%</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
@@ -14383,7 +14411,11 @@
           <t>Students</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Percentage</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -14400,7 +14432,11 @@
       <c r="B11" t="n">
         <v>257</v>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>86%</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
@@ -14417,7 +14453,11 @@
       <c r="B12" t="n">
         <v>9</v>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
@@ -14434,7 +14474,11 @@
       <c r="B13" t="n">
         <v>25</v>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
@@ -14451,7 +14495,11 @@
       <c r="B14" t="n">
         <v>8</v>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
@@ -14468,7 +14516,11 @@
       <c r="B15" t="n">
         <v>0</v>
       </c>
-      <c r="C15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
@@ -14559,7 +14611,7 @@
         <v>159</v>
       </c>
       <c r="C19" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D19" t="n">
         <v>4</v>
@@ -14609,172 +14661,6 @@
       </c>
       <c r="I20" t="n">
         <v>122</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>YEAR-WISE BREAKDOWN</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Department</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Virtual</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>4 Solved</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>3 Solved</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>2 Solved</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>1 Solved</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>0 Solved</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>II Year</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>130</v>
-      </c>
-      <c r="C24" t="n">
-        <v>16</v>
-      </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>III Year</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>114</v>
-      </c>
-      <c r="C25" t="n">
-        <v>27</v>
-      </c>
-      <c r="D25" t="n">
-        <v>2</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" t="n">
-        <v>4</v>
-      </c>
-      <c r="G25" t="n">
-        <v>8</v>
-      </c>
-      <c r="H25" t="n">
-        <v>4</v>
-      </c>
-      <c r="I25" t="n">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>IV Year</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>55</v>
-      </c>
-      <c r="C26" t="n">
-        <v>23</v>
-      </c>
-      <c r="D26" t="n">
-        <v>3</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" t="n">
-        <v>4</v>
-      </c>
-      <c r="G26" t="n">
-        <v>17</v>
-      </c>
-      <c r="H26" t="n">
-        <v>5</v>
-      </c>
-      <c r="I26" t="n">
-        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(sunday-engine): upgrade Sunday Contest GraphQL engine to 10/10 production grade with strict state machine, reconciliation gates, session SHA-256 seal, restart recovery, and 99/99 passing tests
</commit_message>
<xml_diff>
--- a/report_2026-08-09.xlsx
+++ b/report_2026-08-09.xlsx
@@ -3815,11 +3815,7 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E74" t="inlineStr"/>
       <c r="F74" t="b">
         <v>0</v>
       </c>
@@ -3905,11 +3901,7 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E76" t="inlineStr"/>
       <c r="F76" t="b">
         <v>0</v>
       </c>
@@ -4600,11 +4592,7 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E91" t="inlineStr"/>
       <c r="F91" t="b">
         <v>0</v>
       </c>
@@ -5479,11 +5467,7 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E110" t="inlineStr"/>
       <c r="F110" t="b">
         <v>0</v>
       </c>
@@ -5614,11 +5598,7 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E113" t="inlineStr"/>
       <c r="F113" t="b">
         <v>0</v>
       </c>
@@ -5749,11 +5729,7 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E116" t="inlineStr"/>
       <c r="F116" t="b">
         <v>0</v>
       </c>
@@ -6068,11 +6044,7 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E123" t="inlineStr"/>
       <c r="F123" t="b">
         <v>0</v>
       </c>
@@ -6432,11 +6404,7 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E131" t="inlineStr"/>
       <c r="F131" t="b">
         <v>0</v>
       </c>
@@ -6702,11 +6670,7 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E137" t="inlineStr"/>
       <c r="F137" t="b">
         <v>0</v>
       </c>
@@ -8690,11 +8654,7 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E181" t="inlineStr"/>
       <c r="F181" t="b">
         <v>0</v>
       </c>
@@ -8780,11 +8740,7 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E183" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E183" t="inlineStr"/>
       <c r="F183" t="b">
         <v>0</v>
       </c>
@@ -9140,11 +9096,7 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E191" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E191" t="inlineStr"/>
       <c r="F191" t="b">
         <v>0</v>
       </c>
@@ -10644,11 +10596,7 @@
           <t>III</t>
         </is>
       </c>
-      <c r="E223" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E223" t="inlineStr"/>
       <c r="F223" t="b">
         <v>0</v>
       </c>
@@ -11613,11 +11561,7 @@
           <t>III</t>
         </is>
       </c>
-      <c r="E244" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E244" t="inlineStr"/>
       <c r="F244" t="b">
         <v>0</v>
       </c>
@@ -12247,11 +12191,7 @@
           <t>III</t>
         </is>
       </c>
-      <c r="E258" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E258" t="inlineStr"/>
       <c r="F258" t="b">
         <v>0</v>
       </c>
@@ -13167,11 +13107,7 @@
           <t>IV</t>
         </is>
       </c>
-      <c r="E278" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E278" t="inlineStr"/>
       <c r="F278" t="b">
         <v>0</v>
       </c>
@@ -13355,11 +13291,7 @@
           <t>IV</t>
         </is>
       </c>
-      <c r="E282" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E282" t="inlineStr"/>
       <c r="F282" t="b">
         <v>0</v>
       </c>
@@ -13449,11 +13381,7 @@
           <t>IV</t>
         </is>
       </c>
-      <c r="E284" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E284" t="inlineStr"/>
       <c r="F284" t="b">
         <v>0</v>
       </c>
@@ -13678,11 +13606,7 @@
           <t>IV</t>
         </is>
       </c>
-      <c r="E289" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E289" t="inlineStr"/>
       <c r="F289" t="b">
         <v>0</v>
       </c>
@@ -13960,11 +13884,7 @@
           <t>IV</t>
         </is>
       </c>
-      <c r="E295" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E295" t="inlineStr"/>
       <c r="F295" t="b">
         <v>0</v>
       </c>
@@ -14005,11 +13925,7 @@
           <t>IV</t>
         </is>
       </c>
-      <c r="E296" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E296" t="inlineStr"/>
       <c r="F296" t="b">
         <v>0</v>
       </c>

</xml_diff>